<commit_message>
docs: management workbook - tidy verification sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/CKDESK-MANAGEMENT-FEATURE-STATUS.xlsx
+++ b/docs/CKDESK-MANAGEMENT-FEATURE-STATUS.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2636" uniqueCount="1087">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2631" uniqueCount="1083">
   <si>
     <t>CK Desk - what we built, what is live, what is next</t>
   </si>
@@ -2925,18 +2925,6 @@
   </si>
   <si>
     <t>Confirmed</t>
-  </si>
-  <si>
-    <t>WhatsApp and DeskTime</t>
-  </si>
-  <si>
-    <t>Left out of the lists as you asked.</t>
-  </si>
-  <si>
-    <t>-</t>
-  </si>
-  <si>
-    <t>Not listed</t>
   </si>
   <si>
     <t>The live database (10.0.0.205) was NOT queried: that needs the postgres password, which only the owner types. What is configured there (which categories and stores are switched on) comes from the owner. Everything else above was read from the code on main, the live version and health address, and the live app server (services, scheduled task names, setting names with values hidden).</t>
@@ -4052,7 +4040,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="14" t="s">
-        <v>1015</v>
+        <v>1011</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
@@ -4064,33 +4052,33 @@
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="15" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>1013</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>1014</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>1015</v>
+      </c>
+      <c r="E2" s="15" t="s">
         <v>1016</v>
-      </c>
-      <c r="B2" s="15" t="s">
-        <v>1017</v>
-      </c>
-      <c r="C2" s="15" t="s">
-        <v>1018</v>
-      </c>
-      <c r="D2" s="15" t="s">
-        <v>1019</v>
-      </c>
-      <c r="E2" s="15" t="s">
-        <v>1020</v>
       </c>
       <c r="F2" s="15" t="s">
         <v>419</v>
       </c>
       <c r="G2" s="15" t="s">
-        <v>1021</v>
+        <v>1017</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>1022</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>1023</v>
+        <v>1019</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>18</v>
@@ -4108,7 +4096,7 @@
         <v>18</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>18</v>
@@ -4116,7 +4104,7 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>1025</v>
+        <v>1021</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>18</v>
@@ -4134,7 +4122,7 @@
         <v>18</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>18</v>
@@ -4142,7 +4130,7 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>1026</v>
+        <v>1022</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>18</v>
@@ -4160,7 +4148,7 @@
         <v>18</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>18</v>
@@ -4168,7 +4156,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>1027</v>
+        <v>1023</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>18</v>
@@ -4186,7 +4174,7 @@
         <v>18</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>18</v>
@@ -4194,7 +4182,7 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>1028</v>
+        <v>1024</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>18</v>
@@ -4212,7 +4200,7 @@
         <v>18</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>18</v>
@@ -4220,7 +4208,7 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>1029</v>
+        <v>1025</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>18</v>
@@ -4238,7 +4226,7 @@
         <v>18</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>18</v>
@@ -4246,7 +4234,7 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>1030</v>
+        <v>1026</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>18</v>
@@ -4264,7 +4252,7 @@
         <v>18</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>18</v>
@@ -4272,7 +4260,7 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>1031</v>
+        <v>1027</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>18</v>
@@ -4290,7 +4278,7 @@
         <v>18</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>18</v>
@@ -4298,7 +4286,7 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>1032</v>
+        <v>1028</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>18</v>
@@ -4316,7 +4304,7 @@
         <v>18</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H11" s="3" t="s">
         <v>18</v>
@@ -4324,7 +4312,7 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>1033</v>
+        <v>1029</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>18</v>
@@ -4342,7 +4330,7 @@
         <v>18</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>18</v>
@@ -4350,7 +4338,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>1034</v>
+        <v>1030</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>18</v>
@@ -4368,7 +4356,7 @@
         <v>18</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>18</v>
@@ -4376,7 +4364,7 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>1035</v>
+        <v>1031</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>18</v>
@@ -4394,7 +4382,7 @@
         <v>18</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>18</v>
@@ -4402,7 +4390,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>1036</v>
+        <v>1032</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>18</v>
@@ -4420,7 +4408,7 @@
         <v>18</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>18</v>
@@ -4428,7 +4416,7 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>1037</v>
+        <v>1033</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>18</v>
@@ -4446,7 +4434,7 @@
         <v>18</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>18</v>
@@ -4454,7 +4442,7 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>1038</v>
+        <v>1034</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>18</v>
@@ -4472,7 +4460,7 @@
         <v>18</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>1024</v>
+        <v>1020</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>18</v>
@@ -4500,7 +4488,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="20" t="s">
-        <v>1039</v>
+        <v>1035</v>
       </c>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -4508,13 +4496,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="21" t="s">
-        <v>1040</v>
+        <v>1036</v>
       </c>
       <c r="B2" s="21" t="s">
-        <v>1041</v>
+        <v>1037</v>
       </c>
       <c r="C2" s="21" t="s">
-        <v>1042</v>
+        <v>1038</v>
       </c>
       <c r="D2" s="21" t="s">
         <v>605</v>
@@ -4522,27 +4510,27 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="13" t="s">
-        <v>1043</v>
+        <v>1039</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>1044</v>
+        <v>1040</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>1046</v>
+        <v>1042</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>1047</v>
+        <v>1043</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>1048</v>
+        <v>1044</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D4" s="3" t="s">
         <v>18</v>
@@ -4550,13 +4538,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="13" t="s">
-        <v>1049</v>
+        <v>1045</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>1050</v>
+        <v>1046</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>18</v>
@@ -4564,58 +4552,58 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="13" t="s">
-        <v>1051</v>
+        <v>1047</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>1052</v>
+        <v>1048</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>1054</v>
+        <v>1050</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="13" t="s">
-        <v>1055</v>
+        <v>1051</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>1056</v>
+        <v>1052</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>1057</v>
+        <v>1053</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="13" t="s">
-        <v>1058</v>
+        <v>1054</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1059</v>
+        <v>1055</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>1060</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="13" t="s">
-        <v>1061</v>
+        <v>1057</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1062</v>
+        <v>1058</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>1063</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
@@ -4623,38 +4611,38 @@
         <v>453</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1064</v>
+        <v>1060</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>1065</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="13" t="s">
-        <v>1066</v>
+        <v>1062</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>1067</v>
+        <v>1063</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>1068</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="13" t="s">
-        <v>1069</v>
+        <v>1065</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>1070</v>
+        <v>1066</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D12" s="3" t="s">
         <v>18</v>
@@ -4662,16 +4650,16 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="13" t="s">
-        <v>1071</v>
+        <v>1067</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>1072</v>
+        <v>1068</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>1073</v>
+        <v>1069</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
@@ -4679,10 +4667,10 @@
         <v>455</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>1074</v>
+        <v>1070</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D14" s="3" t="s">
         <v>18</v>
@@ -4690,58 +4678,58 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="13" t="s">
-        <v>1075</v>
+        <v>1071</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>1076</v>
+        <v>1072</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>1045</v>
+        <v>1041</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>1077</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="13" t="s">
-        <v>1078</v>
+        <v>1074</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>1079</v>
+        <v>1075</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>1080</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="13" t="s">
-        <v>1081</v>
+        <v>1077</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>1082</v>
+        <v>1078</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>1083</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="13" t="s">
-        <v>1084</v>
+        <v>1080</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>1085</v>
+        <v>1081</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>1053</v>
+        <v>1049</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>1086</v>
+        <v>1082</v>
       </c>
     </row>
   </sheetData>
@@ -12119,7 +12107,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -12660,29 +12648,9 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" s="3">
-        <v>26</v>
-      </c>
-      <c r="B28" s="13" t="s">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>968</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>969</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>970</v>
-      </c>
-      <c r="E28" s="3" t="s">
-        <v>971</v>
-      </c>
-      <c r="F28" s="10" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>972</v>
       </c>
     </row>
   </sheetData>
@@ -12710,7 +12678,7 @@
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>973</v>
+        <v>969</v>
       </c>
       <c r="B1" s="16"/>
       <c r="C1" s="16"/>
@@ -12724,22 +12692,22 @@
         <v>352</v>
       </c>
       <c r="B2" s="17" t="s">
+        <v>970</v>
+      </c>
+      <c r="C2" s="17" t="s">
+        <v>971</v>
+      </c>
+      <c r="D2" s="17" t="s">
+        <v>972</v>
+      </c>
+      <c r="E2" s="17" t="s">
+        <v>973</v>
+      </c>
+      <c r="F2" s="17" t="s">
         <v>974</v>
       </c>
-      <c r="C2" s="17" t="s">
+      <c r="G2" s="17" t="s">
         <v>975</v>
-      </c>
-      <c r="D2" s="17" t="s">
-        <v>976</v>
-      </c>
-      <c r="E2" s="17" t="s">
-        <v>977</v>
-      </c>
-      <c r="F2" s="17" t="s">
-        <v>978</v>
-      </c>
-      <c r="G2" s="17" t="s">
-        <v>979</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -12747,45 +12715,45 @@
         <v>357</v>
       </c>
       <c r="B3" s="3" t="s">
+        <v>976</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>977</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>978</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>979</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>980</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>981</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>982</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>983</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>984</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>985</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="13" t="s">
-        <v>986</v>
+        <v>982</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>987</v>
+        <v>983</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>988</v>
+        <v>984</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>357</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>991</v>
+        <v>987</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
@@ -12793,22 +12761,22 @@
         <v>710</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>992</v>
+        <v>988</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>709</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>357</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>990</v>
+        <v>986</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
@@ -12819,19 +12787,19 @@
         <v>227</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>993</v>
+        <v>989</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>357</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -12839,22 +12807,22 @@
         <v>362</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>996</v>
+        <v>992</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>997</v>
+        <v>993</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="E7" s="3" t="s">
         <v>357</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>998</v>
+        <v>994</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
@@ -12862,22 +12830,22 @@
         <v>379</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>1000</v>
+        <v>996</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>1001</v>
+        <v>997</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>362</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
@@ -12885,22 +12853,22 @@
         <v>383</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>1002</v>
+        <v>998</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>1003</v>
+        <v>999</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>989</v>
+        <v>985</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>1004</v>
+        <v>1000</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>1005</v>
+        <v>1001</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>999</v>
+        <v>995</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
@@ -12908,22 +12876,22 @@
         <v>743</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>1006</v>
+        <v>1002</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>1007</v>
+        <v>1003</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>994</v>
+        <v>990</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>1008</v>
+        <v>1004</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>983</v>
+        <v>979</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>995</v>
+        <v>991</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
@@ -12931,27 +12899,27 @@
         <v>801</v>
       </c>
       <c r="B11" s="3" t="s">
+        <v>1005</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>1008</v>
+      </c>
+      <c r="F11" s="3" t="s">
         <v>1009</v>
       </c>
-      <c r="C11" s="3" t="s">
-        <v>1010</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>1011</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>1012</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>1013</v>
-      </c>
       <c r="G11" s="3" t="s">
-        <v>985</v>
+        <v>981</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>1014</v>
+        <v>1010</v>
       </c>
     </row>
   </sheetData>

</xml_diff>